<commit_message>
Product Book: estado intermediário da reestruturação para o volume do Lodge (em andamento)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MXgeeezmv3d1TAAP83TAQH
</commit_message>
<xml_diff>
--- a/projects/zion-glamping-line/ZION_ORCAMENTO_SC_Casulo_Safari.xlsx
+++ b/projects/zion-glamping-line/ZION_ORCAMENTO_SC_Casulo_Safari.xlsx
@@ -4764,7 +4764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6332,6 +6332,192 @@
         <v>1.2</v>
       </c>
       <c r="G53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>vigota_lsf</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Vigota LSF Ue 150 x 40 x 1,25 galvanizada Z275 (R$/m)</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>21</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F54" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Lodge: módulos de piso e deck</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>hidrofuga</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Membrana hidrófuga + ripas de ventilação da parede (R$/m²)</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>38</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F55" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Lodge: câmara ventilada atrás do ripado</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>lanterna</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Lanterna Ø1,50: vidro laminado curvo 8 + 8 h 0,45 + esquadria RPT + tampa de alumínio (un)</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>12500</v>
+      </c>
+      <c r="E56" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F56" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Lodge; Econ.: policarbonato compacto curvo</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>porta_correr</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Porta de correr de vidro 2,00 x 2,40: trilho embutido, roldanas, puxador, fechadura (un)</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>6500</v>
+      </c>
+      <c r="E57" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F57" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Lodge; folha incluída na fachada</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>vela</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Vela de sombra PVDF ~14 m² confeccionada, com cabos, esticadores e chapas de canto (un)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>6800</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F58" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Lodge; Econ.: tela HDPE 340 g/m²</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>pilar_madeira</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Revestimento de madeira laminada do pilar, 2 meias-canas h 2,70 (un)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>950</v>
+      </c>
+      <c r="E59" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F59" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Lodge; Econ.: pinus autoclavado; Premium: cumaru</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>